<commit_message>
new model data added
</commit_message>
<xml_diff>
--- a/data/benchmark_data.xlsx
+++ b/data/benchmark_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="13920" windowHeight="6732" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="13992" windowHeight="5844" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,19 +16,26 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="165" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="0.000000"/>
-    <numFmt numFmtId="169" formatCode="0.0&quot;%&quot;"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -184,10 +191,6 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
   <fills count="35">
     <fill>
@@ -198,6 +201,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF2563EB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -386,11 +395,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002563EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -406,6 +410,19 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -535,88 +552,72 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="8" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
@@ -631,99 +632,106 @@
     <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1315,272 +1323,334 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.888888888888889" defaultRowHeight="14.4" outlineLevelRow="7"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.888888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.7777777777778" customWidth="1" style="1" min="1" max="1"/>
     <col width="14.6666666666667" customWidth="1" style="1" min="2" max="2"/>
     <col width="8.888888888888889" customWidth="1" style="1" min="3" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" s="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Model </t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
       <c r="C1" s="5" t="n"/>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>MMLU</t>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>MMLU-Pro</t>
         </is>
       </c>
       <c r="E1" s="5" t="n"/>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
       <c r="G1" s="5" t="n"/>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>MMU-PRO</t>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>MMMU-Pro</t>
         </is>
       </c>
       <c r="I1" s="5" t="n"/>
     </row>
-    <row r="2" customFormat="1" s="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="inlineStr">
+    <row r="2" s="1">
+      <c r="A2" s="4" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Rank </t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Score </t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Score </t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Score </t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
     </row>
-    <row r="3" customFormat="1" s="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" s="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro Preview</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="11" t="n">
         <v>94.3</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="11" t="n">
         <v>92.59999999999999</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="E3" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="11" t="n">
         <v>44.4</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="11" t="n">
         <v>80.5</v>
       </c>
-      <c r="I3" s="7" t="n">
+      <c r="I3" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" s="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" s="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Gemini 3.6 Flash</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" customFormat="1" s="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Claude Opus 5</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>93.2</v>
-      </c>
-      <c r="C4" s="7" t="n">
+      <c r="D5" s="11" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" s="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>83</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" s="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Gemma 4 31B</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" s="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Grok 4.20 Reasoning</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>86.59999999999999</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>83.7</v>
+      </c>
+      <c r="I8" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="6" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="E4" s="7" t="n">
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Gemini 3.8 Flash</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>90.221</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="I9" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="6" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>84.7</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" customFormat="1" s="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Gemini 3.6 Flash</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>90.09999999999999</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>83.2</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" customFormat="1" s="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>GPT-5.6 Sol</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>94.59999999999999</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>89.09999999999999</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>83</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" customFormat="1" s="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Gemma 4 31B</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>84.3</v>
-      </c>
-      <c r="C7" s="7" t="n">
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Gpt-5.6 Terra</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" t="n">
+        <v>86.65900000000001</v>
+      </c>
+      <c r="E10" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="E7" s="7" t="n">
+      <c r="F10" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="G10" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="6" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>76.90000000000001</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" customFormat="1" s="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Grok 4.20 Reasoning</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>88.90000000000001</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>86.59999999999999</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>83.7</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>2</v>
+      <c r="H10" s="10" t="n">
+        <v>77</v>
+      </c>
+      <c r="I10" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1600,528 +1670,568 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="20" customWidth="1" style="8" min="1" max="1"/>
-    <col width="28" customWidth="1" style="8" min="2" max="2"/>
-    <col width="12" customWidth="1" style="8" min="3" max="3"/>
-    <col width="100" customWidth="1" style="8" min="4" max="4"/>
+    <col width="20" customWidth="1" style="1" min="1" max="1"/>
+    <col width="28" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="100" customWidth="1" style="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Benchmark</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro Preview</t>
         </is>
       </c>
-      <c r="C2" s="10" t="n">
+      <c r="C2" s="12" t="n">
         <v>94.3</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>Google/OpenAI comparison and secondary benchmark aggregators; no tools.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>MMLU-Pro</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro Preview</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="12" t="n">
         <v>92.59999999999999</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro benchmark reporting; reasoning/high setting.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro Preview</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="12" t="n">
         <v>44.4</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro benchmark reporting; no tools. With-tools result is 51.4%.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>MMMU-Pro</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro Preview</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="12" t="n">
         <v>80.5</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro benchmark reporting; no tools.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="12" t="n">
         <v>93.2</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>Artificial Analysis-derived public snapshot; adaptive reasoning, max effort.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>MMLU-Pro</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="12" t="n">
         <v>91.59999999999999</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Public benchmark aggregation reporting; model-level score.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="12" t="n">
         <v>52.6</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Artificial Analysis-derived public snapshot; adaptive reasoning, max effort.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>MMMU-Pro</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="12" t="n">
         <v>84.7</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Artificial Analysis MMMU-Pro snapshot, July 2026.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.6 Flash</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="12" t="n">
         <v>92.8</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Artificial Analysis-derived public snapshot; high effort.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>MMLU-Pro</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.6 Flash</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="12" t="n">
         <v>90.09999999999999</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Public benchmark comparison source; methodology should be verified before publication.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.6 Flash</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="12" t="n">
         <v>38.3</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Artificial Analysis-derived public snapshot; high effort.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>MMMU-Pro</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>Gemini 3.6 Flash</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="12" t="n">
         <v>83.2</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Artificial Analysis-derived public snapshot.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>GPT-5.6 Sol</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="12" t="n">
         <v>94.59999999999999</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>OpenAI official GPT-5.6 benchmark table.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>MMLU-Pro</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>GPT-5.6 Sol</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="12" t="n">
         <v>89.09999999999999</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>OpenAI official GPT-5.6 benchmark table.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>GPT-5.6 Sol</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="12" t="n">
         <v>47.2</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>OpenAI official GPT-5.6 benchmark table.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>MMMU-Pro</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>GPT-5.6 Sol</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="12" t="n">
         <v>83</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>OpenAI official GPT-5.6 benchmark table; no tools.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>Gemma 4 31B</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="12" t="n">
         <v>84.3</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>Google Gemma 4 model card; no tools.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>MMLU-Pro</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>Gemma 4 31B</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="12" t="n">
         <v>85.2</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>Google Gemma 4 model card.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>Gemma 4 31B</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="12" t="n">
         <v>19.5</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Google Gemma 4 model card; no tools.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>MMMU-Pro</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>Gemma 4 31B</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="12" t="n">
         <v>76.90000000000001</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Google Gemma 4 model card.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>GPQA Diamond</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>Grok 4.20 Reasoning</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C22" s="12" t="n">
         <v>88.90000000000001</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Public Grok 4.20 benchmark summary; reasoning model.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>MMLU-Pro</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>Grok 4.20 Reasoning</t>
         </is>
       </c>
-      <c r="C23" s="10" t="n">
+      <c r="C23" s="12" t="n">
         <v>86.59999999999999</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>Public Grok 4.20 benchmark summary.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>Grok 4.20 Reasoning</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="12" t="n">
         <v>32.2</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Public Grok 4.20 benchmark comparison; exact benchmark harness should be verified before publication.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>MMMU-Pro</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>Grok 4.20 Reasoning</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="C25" s="12" t="n">
         <v>83.7</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>AgMoDB July 2026 leaderboard, Grok 4.20 0309 reasoning.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>Methodology</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" s="10" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr"/>
+      <c r="C26" s="12" t="inlineStr"/>
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>Scores are displayed as reported percentages. Ranks in Sheet1 are calculated only within the six selected models. Public benchmark harness/settings differ across sources, so values should be treated as contextual comparisons rather than a single controlled head-to-head experiment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MMLU-Pro</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gemini 3.8 Flash</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>90.221</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Vals AI-derived public benchmark comparison; score reported as 90.221%. Web source: Gradually.ai benchmark comparison, accessed 2026-09-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MMLU-Pro</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Terra</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>86.65900000000001</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Vals AI-derived public benchmark comparison; score reported as 86.659%. Web source: Gradually.ai benchmark comparison, accessed 2026-09-08.</t>
         </is>
       </c>
     </row>

</xml_diff>